<commit_message>
Update teachers_latest.xlsx (2026-03-28 02:47:16)
</commit_message>
<xml_diff>
--- a/incoming/teachers_latest.xlsx
+++ b/incoming/teachers_latest.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="template" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="teachers" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -43,7 +43,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -51,13 +51,23 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D9E1F2"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,14 +433,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -439,70 +445,200 @@
           <t>teacher_name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>department</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>position</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>trios_url</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>manual_research_fields</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>山田太郎</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>社会工学学位プログラム</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>教授</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>最適化;意思決定支援</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>吉瀬章子</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>鈴木花子</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>社会工学学位プログラム</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>准教授</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>需要予測;物流最適化</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>小西葉子</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>高野祐一</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>繆瑩</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>有馬澄佳</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>イリチュ美佳</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>志田洋平</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>大久保正勝</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Phung-DucTuan</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>張勇兵</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>岡田幸彦</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>上市秀雄</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>黒瀬雄大</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>佐野幸恵</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>秋山英三</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>TranLamAnhDuong</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>LiuTianxiang</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>奥島真一郎</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>八森正泰</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>原田信行</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>藤井さやか</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>繁野麻衣子</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>木下陽平</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>讃井知</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>作道真理</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>髙橋裕紀</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>大西正輝</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>岡本直久</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update teachers_latest.xlsx (2026-03-29 20:54:09)
</commit_message>
<xml_diff>
--- a/incoming/teachers_latest.xlsx
+++ b/incoming/teachers_latest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\takum\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6284149C-5E02-450E-AB47-96AE86215986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CEFA923-DA32-40AF-807F-35C1AC861746}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6825" yWindow="4350" windowWidth="11010" windowHeight="8190" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -73,9 +73,6 @@
     <t>八森正泰</t>
   </si>
   <si>
-    <t>原田信行</t>
-  </si>
-  <si>
     <t>藤井さやか</t>
   </si>
   <si>
@@ -109,6 +106,10 @@
   </si>
   <si>
     <t>Liu Tianxiang</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>原田信行</t>
     <phoneticPr fontId="2"/>
   </si>
 </sst>
@@ -537,7 +538,7 @@
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A10" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.15">
@@ -572,12 +573,12 @@
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A17" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A18" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.15">
@@ -592,47 +593,47 @@
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A21" s="2" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A22" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A23" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A24" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A25" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A26" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A27" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A28" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A29" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update teachers_latest.xlsx (2026-07-04 21:59:38)
</commit_message>
<xml_diff>
--- a/incoming/teachers_latest.xlsx
+++ b/incoming/teachers_latest.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\takum\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC4DD0E5-2E5D-4ED4-A329-3736F6A3EE19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F49FACE-7FC8-4601-A45E-CFB1DD509043}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11415" yWindow="0" windowWidth="11730" windowHeight="14745" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="23280" windowHeight="14880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="指導教員一覧" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="50">
   <si>
     <t>No.</t>
   </si>
@@ -35,9 +35,6 @@
     <t>牛島 光一</t>
   </si>
   <si>
-    <t>MPPS</t>
-  </si>
-  <si>
     <t>藤川 昌樹</t>
   </si>
   <si>
@@ -120,9 +117,6 @@
   </si>
   <si>
     <t>岡田 幸彦</t>
-  </si>
-  <si>
-    <t>MSE</t>
   </si>
   <si>
     <t>志田 洋平</t>
@@ -493,7 +487,7 @@
         <v>3</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -501,10 +495,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -512,10 +506,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -523,10 +517,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -534,10 +528,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -545,10 +539,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -556,10 +550,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -567,10 +561,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -578,10 +572,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -589,10 +583,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -600,10 +594,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -611,10 +605,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -622,10 +616,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -633,10 +627,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -644,10 +638,10 @@
         <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -655,10 +649,10 @@
         <v>16</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -666,10 +660,10 @@
         <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -677,10 +671,10 @@
         <v>18</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -688,10 +682,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -699,10 +693,10 @@
         <v>20</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -710,10 +704,10 @@
         <v>21</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -721,10 +715,10 @@
         <v>22</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -732,10 +726,10 @@
         <v>23</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -743,10 +737,10 @@
         <v>24</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -754,10 +748,10 @@
         <v>25</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -765,10 +759,10 @@
         <v>26</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -776,10 +770,10 @@
         <v>27</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -787,10 +781,10 @@
         <v>28</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -798,10 +792,10 @@
         <v>29</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>33</v>
+        <v>8</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -809,10 +803,10 @@
         <v>30</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>33</v>
+        <v>8</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -820,10 +814,10 @@
         <v>31</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>33</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -846,37 +840,37 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15">
       <c r="A1" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B5">
         <v>107</v>
@@ -884,7 +878,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B6">
         <v>115</v>
@@ -892,7 +886,7 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B7">
         <v>31</v>
@@ -900,7 +894,7 @@
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B8">
         <v>22</v>
@@ -908,7 +902,7 @@
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B9">
         <v>3</v>
@@ -916,7 +910,7 @@
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B10">
         <v>6</v>
@@ -924,10 +918,10 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B11" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>